<commit_message>
Change fuel price of coal for scen 2
</commit_message>
<xml_diff>
--- a/VerveStacks_EST/SuppXLS/Scen_base2.xlsx
+++ b/VerveStacks_EST/SuppXLS/Scen_base2.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\Admin\PycharmProjects\ee-times\VerveStacks_EST\SuppXLS\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{AE63942A-84F0-4BC7-8B18-28256E34928E}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{C909134C-35B3-4AB6-AC34-051AD30D5DF8}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-110" yWindow="-110" windowWidth="19420" windowHeight="11500" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Co2" sheetId="1" r:id="rId1"/>
@@ -478,7 +478,7 @@
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{13560296-7955-4D55-8E7E-094E43148A2D}">
-  <dimension ref="A2:I7"/>
+  <dimension ref="A2:I10"/>
   <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
   <cols>
     <col min="1" max="1" width="27.90625" bestFit="1" customWidth="1"/>
@@ -557,30 +557,30 @@
       <c r="B5" t="s">
         <v>10</v>
       </c>
-      <c r="C5" s="1">
-        <v>96.367112810707454</v>
-      </c>
-      <c r="D5" s="1">
-        <v>96.367112810707454</v>
+      <c r="C5">
+        <v>60</v>
+      </c>
+      <c r="D5">
+        <v>60</v>
       </c>
       <c r="E5" s="1">
-        <f>D5+(D5*0.03)</f>
+        <f>D10+(D10*0.03)</f>
         <v>99.25812619502868</v>
       </c>
       <c r="F5" s="1">
-        <f>E5+(E5*0.03)</f>
+        <f t="shared" ref="E5:I6" si="0">E5+(E5*0.03)</f>
         <v>102.23586998087954</v>
       </c>
       <c r="G5" s="1">
-        <f>F5+(F5*0.03)</f>
+        <f t="shared" si="0"/>
         <v>105.30294608030593</v>
       </c>
       <c r="H5" s="1">
-        <f>G5+(G5*0.03)</f>
+        <f t="shared" si="0"/>
         <v>108.46203446271511</v>
       </c>
       <c r="I5" s="1">
-        <f>H5+(H5*0.03)</f>
+        <f t="shared" si="0"/>
         <v>111.71589549659656</v>
       </c>
     </row>
@@ -598,23 +598,23 @@
         <v>46.470588235294123</v>
       </c>
       <c r="E6" s="1">
-        <f>D6+(D6*0.03)</f>
+        <f t="shared" si="0"/>
         <v>47.864705882352943</v>
       </c>
       <c r="F6" s="1">
-        <f>E6+(E6*0.03)</f>
+        <f t="shared" si="0"/>
         <v>49.300647058823529</v>
       </c>
       <c r="G6" s="1">
-        <f>F6+(F6*0.03)</f>
+        <f t="shared" si="0"/>
         <v>50.779666470588232</v>
       </c>
       <c r="H6" s="1">
-        <f>G6+(G6*0.03)</f>
+        <f t="shared" si="0"/>
         <v>52.303056464705882</v>
       </c>
       <c r="I6" s="1">
-        <f>H6+(H6*0.03)</f>
+        <f t="shared" si="0"/>
         <v>53.872148158647057</v>
       </c>
     </row>
@@ -650,6 +650,14 @@
       <c r="I7" s="1">
         <f>H7+(H7*0.02)</f>
         <v>43.081824438374397</v>
+      </c>
+    </row>
+    <row r="10" spans="1:9" x14ac:dyDescent="0.35">
+      <c r="C10" s="1">
+        <v>96.367112810707454</v>
+      </c>
+      <c r="D10" s="1">
+        <v>96.367112810707454</v>
       </c>
     </row>
   </sheetData>

</xml_diff>